<commit_message>
EPBDS-15725 Remove the deprecated JSON helpers and Jackson typing options
</commit_message>
<xml_diff>
--- a/STUDIO/org.openl.rules.project.validation.openapi/test-resources/functionality/EPBDS-10351_SpreadsheetResult_CastingCells_Convertation.xlsx
+++ b/STUDIO/org.openl.rules.project.validation.openapi/test-resources/functionality/EPBDS-10351_SpreadsheetResult_CastingCells_Convertation.xlsx
@@ -33,7 +33,7 @@
     <t>import</t>
   </si>
   <si>
-    <t>org.openl.rules.serialization.JsonUtils</t>
+    <t>org.openl.rules.serialization.JacksonObjectMapperFactoryBean</t>
   </si>
   <si>
     <t>Spreadsheet SpreadsheetResult Calc()</t>
@@ -189,7 +189,7 @@
     <t>Step3</t>
   </si>
   <si>
-    <t>= JsonUtils.toJSON($Step1)</t>
+    <t>= new JacksonObjectMapperFactoryBean().createJacksonObjectMapper().writeValueAsString($Step1)</t>
   </si>
   <si>
     <t>Step4</t>
@@ -201,7 +201,7 @@
     <t>= Calc2($Step4)</t>
   </si>
   <si>
-    <t>= (SpreadsheetResult) JsonUtils.fromJSON($Step3, SpreadsheetResult.class)</t>
+    <t>= (SpreadsheetResult) new JacksonObjectMapperFactoryBean().createJacksonObjectMapper().readValue($Step3, SpreadsheetResult.class)</t>
   </si>
   <si>
     <t>Test Calc3 Calc3Test</t>

</xml_diff>